<commit_message>
Refinment, new areas added
</commit_message>
<xml_diff>
--- a/expert-system/output/accounting/accounting.xlsx
+++ b/expert-system/output/accounting/accounting.xlsx
@@ -16,6 +16,7 @@
     <sheet name="TS-ACC-Views" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="TS-ACC-SickLeave" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="TS-ACC-APIErrors" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Test Data" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Risk Assessment'!$A$4:$F$19</definedName>
@@ -33,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,8 +86,12 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +140,12 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+        <bgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -162,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,6 +206,16 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -561,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -799,6 +820,13 @@
       </c>
       <c r="D18" s="11" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Test Data Reference</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId1"/>
@@ -807,6 +835,737 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId7"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00BF8F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Accounting Module Test Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>&lt;- Back to Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>1. Recommended Test Users (Module-Specific)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>User / Query</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Roles</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Use Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Use ilnitsky or ann</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>ACCOUNTANT+ADMIN</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Period management and vacation payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Use perekrest</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>CHIEF_ACCOUNTANT</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Chief accountant operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>2. Common Multi-Role Test Users (All Modules)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Roles</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Best For</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>perekrest</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>ACCOUNTANT, ADMIN, CHIEF_ACCOUNTANT, DEPT_MGR, EMPLOYEE, HR, PM</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Best multi-role user (7 roles). Use for cross-role permission testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>pvaynmaster</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>ACCOUNTANT, ADMIN, CHIEF_OFFICER, DEPT_MGR, EMPLOYEE, HR, PM</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Multi-role with CHIEF_OFFICER. Use for highest-privilege scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>ilnitsky</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>ACCOUNTANT, ADMIN, DEPT_MGR, EMPLOYEE, HR, PM</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Admin+accountant combo. Use for accounting and admin tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>ann</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>ACCOUNTANT, ADMIN, DEPT_MGR, EMPLOYEE, HR, PM</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Same role set as ilnitsky. Use as second admin/accountant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>juliet_nekhor</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>DEPT_MGR, EMPLOYEE, HR, PM, VIEW_ALL</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Has VIEW_ALL. Use for read-only permission tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>kcherenkov</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>DEPT_MGR, EMPLOYEE, PM, TECH_LEAD</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Tech Lead + PM. Use for planner/project management tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>alsmirnov</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>EMPLOYEE</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>EMPLOYEE-only. Use as minimum-privilege baseline user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>3. Common SQL Queries (User Discovery)</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>SQL Query</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Find EMPLOYEE-only users (minimum privilege)</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>SELECT e.login, e.full_name
+FROM employee e
+JOIN employee_global_roles r ON e.id = r.employee_id
+WHERE e.enabled = true
+GROUP BY e.id
+HAVING COUNT(*) = 1 AND MAX(r.role) = 'ROLE_EMPLOYEE'
+LIMIT 5;</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>ttt_backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Find active contractors</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>SELECT e.login, e.full_name
+FROM employee e
+JOIN employee_global_roles r ON e.id = r.employee_id
+WHERE e.enabled = true AND r.role = 'ROLE_CONTRACTOR'
+LIMIT 5;</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>ttt_backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Find active project managers</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>SELECT e.login, e.full_name
+FROM employee e
+JOIN employee_global_roles r ON e.id = r.employee_id
+WHERE e.enabled = true AND r.role = 'ROLE_PROJECT_MANAGER'
+LIMIT 5;</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>ttt_backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Find active accountants</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>SELECT e.login, e.full_name
+FROM employee e
+JOIN employee_global_roles r ON e.id = r.employee_id
+WHERE e.enabled = true AND r.role = 'ROLE_ACCOUNTANT'
+LIMIT 5;</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>ttt_backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Find active admins</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>SELECT e.login, e.full_name
+FROM employee e
+JOIN employee_global_roles r ON e.id = r.employee_id
+WHERE e.enabled = true AND r.role = 'ROLE_ADMIN'
+LIMIT 5;</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>ttt_backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Get current report/approve periods per office</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>SELECT o.id as office_id, o.name,
+       rp.start as report_period_start,
+       ap.start as approve_period_start
+FROM office o
+JOIN office_period rp ON o.report_period_id = rp.id
+JOIN office_period ap ON o.approve_period_id = ap.id
+ORDER BY o.id;</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>ttt</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>4. Module-Specific SQL Queries</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>SQL Query</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Find offices with current period state</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>SELECT o.id, o.name,
+       rp.start as report_start, ap.start as approve_start
+FROM ttt_backend.office o
+JOIN ttt_backend.office_period rp ON o.report_period_id = rp.id
+JOIN ttt_backend.office_period ap ON o.approve_period_id = ap.id
+ORDER BY o.id;</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Run on timemachine/qa-1 DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Find APPROVED vacations available for payment</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>SELECT v.id, v.login, v.start_date, v.end_date, v.payment_type, v.days
+FROM ttt_vacation.vacation v
+WHERE v.status = 'APPROVED'
+ORDER BY v.start_date LIMIT 20;</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Run on timemachine/qa-1 DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Find employees with vacation day corrections</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>SELECT vdc.id, vdc.employee_login, vdc.days, vdc.year, vdc.reason
+FROM ttt_vacation.vacation_day_correction vdc
+ORDER BY vdc.id DESC LIMIT 20;</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Run on timemachine/qa-1 DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Find office norm data for period validation</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>SELECT sr.employee_login, sr.date, sr.norm, sr.reported
+FROM ttt_backend.statistic_report sr
+WHERE sr.date &gt;= '2026-03-01'
+ORDER BY sr.employee_login, sr.date LIMIT 30;</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Run on timemachine/qa-1 DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>5. Data Generation Strategies</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Period dates</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Format: YYYY-MM-01 (always 1st of month). Advance: current start + 1 month. Revert: current start - 1 month.</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>officeId</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Use offices 2 (Saturn), 10 (Venus), 4 (Jupiter) — largest offices. Avoid office 9 (stuck at 2020-03-01).</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Payment validation</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Payment requires: status=APPROVED, startDate in approved period, 5 business checks pass. Use APPROVED vacations from query above.</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Day correction</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>days field accepts positive (add) and negative (subtract). Boundary: 0 (no-op), large negative &gt; available (expect error).</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>6. Environment Reference</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="11" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>timemachine</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>https://ttt-timemachine.noveogroup.com</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Primary dev env — has test clock (PATCH to advance time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>qa-1</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>https://ttt-qa-1.noveogroup.com</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Secondary dev env — real clock</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>stage</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>https://ttt-stage.noveogroup.com</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Production-like env — read-only testing preferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>7. API Authentication</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="11" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>How to Obtain/Use</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>JWT (user context)</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Login via CAS SSO at /login, extract TTT_JWT_TOKEN cookie. Pass as Authorization: Bearer &lt;token&gt; or Cookie header.</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Most endpoints</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>API token</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Set header API_SECRET_TOKEN: &lt;token_value&gt;. Value from env config file.</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Test/sync endpoints, limited scope</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A48:C48"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>